<commit_message>
Fixed a bug in plotting the dose response. Added a new application on Oscillators (still testing).
</commit_message>
<xml_diff>
--- a/apps_results_MAK_REINFORCE/RPA_2species_4rxns/RPA_2species_4rxns_MAK_REINFORCE.xlsx
+++ b/apps_results_MAK_REINFORCE/RPA_2species_4rxns/RPA_2species_4rxns_MAK_REINFORCE.xlsx
@@ -10,14 +10,14 @@
     <sheet r:id="rId1" sheetId="1" name="Data"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$W$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$W$5</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>Timestamp</t>
   </si>
@@ -88,22 +88,22 @@
     <t>Structure Head Temperature</t>
   </si>
   <si>
-    <t>2025-11-24 16:11:38</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/8a51c6a6eaf542a08f29b145f907076d</t>
-  </si>
-  <si>
-    <t>No</t>
+    <t>2025-11-25 00:24:05</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/dd9684eec8294297ab7ac5291901cdb5</t>
+  </si>
+  <si>
+    <t>Yes*</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Didn't have enough epochs, but it looked like it was converging.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+    <t>Decreased the global entorpy weight a bit. Seems to yield some topologies.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.003, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
     <t>0.0001</t>
@@ -121,109 +121,28 @@
     <t>{'target_entropy_ratio_to_max': np.float64(0.4686790650623293), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
   </si>
   <si>
-    <t>2025-11-24 17:31:46</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/1e46196e688e4a0d9615b43e07ea4cff</t>
-  </si>
-  <si>
-    <t>Increased the number of epochs. Converged quickly but not to a value low enough.</t>
-  </si>
-  <si>
-    <t>2025-11-24 18:23:00</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/29ee16bcf9264cef81c3d3b36a4a2a7d</t>
-  </si>
-  <si>
-    <t>Yes?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decreased the entropy weight of the parameter head. </t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-24 18:59:21</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/cc0eb6ffd82e487886169efe71e77835</t>
-  </si>
-  <si>
-    <t>Decreased the entropy weight of the parameter head even more. Seemed to increase generative power.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-24 19:51:57</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/8f4fdcf082444cd182e0b8d6544ad8d3</t>
-  </si>
-  <si>
-    <t>Increased the global entropy weight. Diverged.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.005, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-25 00:24:05</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/dd9684eec8294297ab7ac5291901cdb5</t>
-  </si>
-  <si>
-    <t>Yes*</t>
-  </si>
-  <si>
-    <t>Decreased the global entorpy weight a bit. Seems to yield some topologies.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.003, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-25 09:10:20</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/2bfc929bd1b24cf482692b4d6cd7b79a</t>
-  </si>
-  <si>
-    <t>Yes/No</t>
-  </si>
-  <si>
-    <t>Same conditions as previous run. Got one topology only.</t>
-  </si>
-  <si>
-    <t>2025-11-25 10:32:00</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/88f51f676edf4498b8af94be2cd85fe2</t>
-  </si>
-  <si>
-    <t>Same conditions as previous run. Got one topology only, but it seemed that it was exploring.</t>
-  </si>
-  <si>
-    <t>2025-11-25 11:07:37</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/8e6ab6524baa4196a676973ccfe42b76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Increased the entropy weight of the structure head a bit. </t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.004, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
     <t>2025-11-25 15:42:18</t>
   </si>
   <si>
     <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/5facc08760b449f187c3c2069a356902</t>
   </si>
   <si>
-    <t>Same as row 7.</t>
+    <t>Same as before. Good run.</t>
+  </si>
+  <si>
+    <t>2025-11-25 16:05:21</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/8b2f389fd2c84a1597e3e2f96dd1e7e2</t>
+  </si>
+  <si>
+    <t>Same as before.</t>
+  </si>
+  <si>
+    <t>2025-11-26 08:50:20</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-2species-4rxns-mak-reinforce/a1380413479149a29cc4ffb504edf0e1</t>
   </si>
 </sst>
 </file>
@@ -598,7 +517,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
@@ -606,7 +525,7 @@
     <col min="3" max="3" style="4" width="11.005" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="4" width="17.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="4" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="99.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="75.005" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="4" width="254.005" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="4" width="14.005" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="5" width="9.005" customWidth="1" bestFit="1"/>
@@ -711,7 +630,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>27</v>
@@ -723,7 +642,7 @@
         <v>29</v>
       </c>
       <c r="I2" s="2">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>30</v>
@@ -782,7 +701,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>36</v>
@@ -847,7 +766,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>26</v>
@@ -856,10 +775,10 @@
         <v>26</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>29</v>
@@ -910,15 +829,15 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>26</v>
@@ -927,477 +846,57 @@
         <v>26</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="3">
         <v>300</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="3">
         <v>5</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="3">
         <v>1024</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="3">
         <v>10240</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="3">
         <v>128</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="3">
         <v>10</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="3">
         <v>30</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="3">
         <v>100</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="3">
         <v>1000</v>
       </c>
-      <c r="T5" s="2">
+      <c r="T5" s="3">
         <v>1</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="3">
         <v>9</v>
       </c>
       <c r="V5" s="1" t="s">
         <v>32</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="2">
-        <v>300</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="2">
-        <v>5</v>
-      </c>
-      <c r="L6" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M6" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N6" s="2">
-        <v>128</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>30</v>
-      </c>
-      <c r="R6" s="2">
-        <v>100</v>
-      </c>
-      <c r="S6" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T6" s="2">
-        <v>1</v>
-      </c>
-      <c r="U6" s="2">
-        <v>9</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="2">
-        <v>300</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="2">
-        <v>5</v>
-      </c>
-      <c r="L7" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M7" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N7" s="2">
-        <v>128</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>30</v>
-      </c>
-      <c r="R7" s="2">
-        <v>100</v>
-      </c>
-      <c r="S7" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T7" s="2">
-        <v>1</v>
-      </c>
-      <c r="U7" s="2">
-        <v>9</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I8" s="2">
-        <v>300</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8" s="2">
-        <v>5</v>
-      </c>
-      <c r="L8" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M8" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N8" s="2">
-        <v>128</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P8" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="2">
-        <v>30</v>
-      </c>
-      <c r="R8" s="2">
-        <v>100</v>
-      </c>
-      <c r="S8" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T8" s="2">
-        <v>1</v>
-      </c>
-      <c r="U8" s="2">
-        <v>9</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="2">
-        <v>300</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="2">
-        <v>5</v>
-      </c>
-      <c r="L9" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M9" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N9" s="2">
-        <v>128</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P9" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q9" s="2">
-        <v>30</v>
-      </c>
-      <c r="R9" s="2">
-        <v>100</v>
-      </c>
-      <c r="S9" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T9" s="2">
-        <v>1</v>
-      </c>
-      <c r="U9" s="2">
-        <v>9</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I10" s="2">
-        <v>300</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K10" s="2">
-        <v>5</v>
-      </c>
-      <c r="L10" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M10" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N10" s="2">
-        <v>128</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P10" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q10" s="2">
-        <v>30</v>
-      </c>
-      <c r="R10" s="2">
-        <v>100</v>
-      </c>
-      <c r="S10" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T10" s="2">
-        <v>1</v>
-      </c>
-      <c r="U10" s="2">
-        <v>9</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
-      <c r="A11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I11" s="3">
-        <v>300</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K11" s="3">
-        <v>5</v>
-      </c>
-      <c r="L11" s="3">
-        <v>1024</v>
-      </c>
-      <c r="M11" s="3">
-        <v>10240</v>
-      </c>
-      <c r="N11" s="3">
-        <v>128</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P11" s="3">
-        <v>10</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>30</v>
-      </c>
-      <c r="R11" s="3">
-        <v>100</v>
-      </c>
-      <c r="S11" s="3">
-        <v>1000</v>
-      </c>
-      <c r="T11" s="3">
-        <v>1</v>
-      </c>
-      <c r="U11" s="3">
-        <v>9</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W11" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>